<commit_message>
feat(stories): refine member experience submission
</commit_message>
<xml_diff>
--- a/public/downloads/sample-ipace-owner-data.xlsx
+++ b/public/downloads/sample-ipace-owner-data.xlsx
@@ -12,13 +12,20 @@
     <sheet name="Vehicles" sheetId="3" r:id="rId5"/>
     <sheet name="SoH History" sheetId="4" r:id="rId6"/>
     <sheet name="Service &amp; Faults" sheetId="5" r:id="rId7"/>
+    <sheet name="Experiences" sheetId="6" r:id="rId8"/>
   </sheets>
+  <definedNames>
+    <definedName hidden="true" localSheetId="1" name="_xlnm._FilterDatabase">'Membership'!$A$1:$M$2</definedName>
+    <definedName hidden="true" localSheetId="2" name="_xlnm._FilterDatabase">'Vehicles'!$A$1:$N$3</definedName>
+    <definedName hidden="true" localSheetId="3" name="_xlnm._FilterDatabase">'SoH History'!$A$1:$G$6</definedName>
+    <definedName hidden="true" localSheetId="4" name="_xlnm._FilterDatabase">'Service &amp; Faults'!$A$1:$AA$5</definedName>
+  </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
   <si>
     <t>My I-PACE owner data</t>
   </si>
@@ -47,6 +54,9 @@
     <t>Service and fault events</t>
   </si>
   <si>
+    <t>Member experiences</t>
+  </si>
+  <si>
     <t>This workbook is a portable copy of the data currently saved in your member account. It excludes internal identity and security hashes.</t>
   </si>
   <si>
@@ -83,6 +93,15 @@
     <t>Skills</t>
   </si>
   <si>
+    <t>Willing to help</t>
+  </si>
+  <si>
+    <t>Expertise</t>
+  </si>
+  <si>
+    <t>Press story</t>
+  </si>
+  <si>
     <t>Contact consent</t>
   </si>
   <si>
@@ -110,6 +129,12 @@
     <t>Community support; Technical</t>
   </si>
   <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>true</t>
   </si>
   <si>
@@ -275,6 +300,21 @@
     <t>Dispute status</t>
   </si>
   <si>
+    <t>Executive Office acknowledgement</t>
+  </si>
+  <si>
+    <t>Executive Office reply</t>
+  </si>
+  <si>
+    <t>Executive Office outcome</t>
+  </si>
+  <si>
+    <t>Satisfied with outcome</t>
+  </si>
+  <si>
+    <t>JLR Client Care case reference</t>
+  </si>
+  <si>
     <t>2025-11-14</t>
   </si>
   <si>
@@ -323,9 +363,6 @@
     <t>Complete</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Not applicable</t>
   </si>
   <si>
@@ -357,6 +394,54 @@
   </si>
   <si>
     <t>Diagnostic report added to personal records.</t>
+  </si>
+  <si>
+    <t>Editorial title</t>
+  </si>
+  <si>
+    <t>Published name</t>
+  </si>
+  <si>
+    <t>Experience (Markdown)</t>
+  </si>
+  <si>
+    <t>Linked service and JLR records</t>
+  </si>
+  <si>
+    <t>Linked SoH readings</t>
+  </si>
+  <si>
+    <t>Executive Office contacts</t>
+  </si>
+  <si>
+    <t>Website permission</t>
+  </si>
+  <si>
+    <t>Third-party permission</t>
+  </si>
+  <si>
+    <t>Copyright confirmed</t>
+  </si>
+  <si>
+    <t>Truthful confirmed</t>
+  </si>
+  <si>
+    <t>Consent version</t>
+  </si>
+  <si>
+    <t>Consent recorded</t>
+  </si>
+  <si>
+    <t>Member message</t>
+  </si>
+  <si>
+    <t>Media count</t>
+  </si>
+  <si>
+    <t>Media names</t>
+  </si>
+  <si>
+    <t>Published</t>
   </si>
 </sst>
 </file>
@@ -427,7 +512,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment vertical="center"/>
@@ -440,6 +525,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true" applyAlignment="false">
+      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -958,95 +1046,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MembershipTable" displayName="MembershipTable" ref="A1:J2">
-  <autoFilter ref="A1:J2"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="Email"/>
-    <tableColumn id="2" name="Name"/>
-    <tableColumn id="3" name="Country"/>
-    <tableColumn id="4" name="Relationship"/>
-    <tableColumn id="5" name="Skills"/>
-    <tableColumn id="6" name="Contact consent"/>
-    <tableColumn id="7" name="Anonymised analysis"/>
-    <tableColumn id="8" name="Participation acknowledged"/>
-    <tableColumn id="9" name="Joined"/>
-    <tableColumn id="10" name="Updated"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="false" showLastColumn="false" showRowStripes="true" showColumnStripes="false"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="VehiclesTable" displayName="VehiclesTable" ref="A1:N3">
-  <autoFilter ref="A1:N3"/>
-  <tableColumns count="14">
-    <tableColumn id="1" name="Vehicle"/>
-    <tableColumn id="2" name="Registration"/>
-    <tableColumn id="3" name="VIN last 6"/>
-    <tableColumn id="4" name="Country"/>
-    <tableColumn id="5" name="Model year"/>
-    <tableColumn id="6" name="Mileage"/>
-    <tableColumn id="7" name="Owned since"/>
-    <tableColumn id="8" name="First registered"/>
-    <tableColumn id="9" name="Latest SoH %"/>
-    <tableColumn id="10" name="SoH measured"/>
-    <tableColumn id="11" name="SoH mileage"/>
-    <tableColumn id="12" name="SoH source"/>
-    <tableColumn id="13" name="Created"/>
-    <tableColumn id="14" name="Updated"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="false" showLastColumn="false" showRowStripes="true" showColumnStripes="false"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SoHHistoryTable" displayName="SoHHistoryTable" ref="A1:G6">
-  <autoFilter ref="A1:G6"/>
-  <tableColumns count="7">
-    <tableColumn id="1" name="Vehicle"/>
-    <tableColumn id="2" name="Measured"/>
-    <tableColumn id="3" name="State of health %"/>
-    <tableColumn id="4" name="Mileage"/>
-    <tableColumn id="5" name="Source"/>
-    <tableColumn id="6" name="Recorded"/>
-    <tableColumn id="7" name="Updated"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="false" showLastColumn="false" showRowStripes="true" showColumnStripes="false"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ServiceAndFaultsTable" displayName="ServiceAndFaultsTable" ref="A1:V5">
-  <autoFilter ref="A1:V5"/>
-  <tableColumns count="22">
-    <tableColumn id="1" name="Vehicle"/>
-    <tableColumn id="2" name="Type"/>
-    <tableColumn id="3" name="Date"/>
-    <tableColumn id="4" name="Mileage"/>
-    <tableColumn id="5" name="Title"/>
-    <tableColumn id="6" name="Description"/>
-    <tableColumn id="7" name="Status"/>
-    <tableColumn id="8" name="Campaigns"/>
-    <tableColumn id="9" name="Service provider"/>
-    <tableColumn id="10" name="Provider postcode"/>
-    <tableColumn id="11" name="Authorised JLR provider"/>
-    <tableColumn id="12" name="Final fix date"/>
-    <tableColumn id="13" name="Days to final fix"/>
-    <tableColumn id="14" name="Courtesy vehicle offered"/>
-    <tableColumn id="15" name="Courtesy vehicle provided"/>
-    <tableColumn id="16" name="Parts delay"/>
-    <tableColumn id="17" name="Goodwill payment"/>
-    <tableColumn id="18" name="Miles driven whilst faulty"/>
-    <tableColumn id="19" name="Warranty cover"/>
-    <tableColumn id="20" name="Dispute status"/>
-    <tableColumn id="21" name="Created"/>
-    <tableColumn id="22" name="Updated"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="false" showLastColumn="false" showRowStripes="true" showColumnStripes="false"/>
-</table>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -1324,15 +1323,15 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="J1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2">
       <c r="J2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1346,7 +1345,7 @@
         <v>2</v>
       </c>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K3">
         <v>1</v>
@@ -1360,7 +1359,7 @@
         <v>4</v>
       </c>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K4">
         <v>1</v>
@@ -1369,7 +1368,7 @@
     <row r="5">
       <c r="A5" s="3"/>
       <c r="J5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -1407,9 +1406,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
     <row r="12" ht="24" customHeight="true">
       <c r="A12" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" s="4"/>
     </row>
@@ -1432,84 +1439,102 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="10" min="1" width="18"/>
+    <col customWidth="true" max="13" min="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="true">
       <c r="A1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="B2" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="C2" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J2" t="s">
-        <v>31</v>
+      <c r="D2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
+  <autoFilter ref="$A$1:$M$2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
     <col customWidth="true" max="14" min="1" width="18"/>
@@ -1517,145 +1542,144 @@
   <sheetData>
     <row r="1" ht="30" customHeight="true">
       <c r="A1" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="5">
+        <v>48520</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="I2" s="5">
+        <v>88.4</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" s="5">
+        <v>48380</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="M2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F2">
-        <v>48520</v>
-      </c>
-      <c r="G2" t="s">
-        <v>47</v>
-      </c>
-      <c r="H2" t="s">
-        <v>48</v>
-      </c>
-      <c r="I2">
-        <v>88.4</v>
-      </c>
-      <c r="J2" t="s">
-        <v>49</v>
-      </c>
-      <c r="K2">
-        <v>48380</v>
-      </c>
-      <c r="L2" t="s">
-        <v>50</v>
-      </c>
-      <c r="M2" t="s">
-        <v>31</v>
-      </c>
-      <c r="N2" t="s">
-        <v>51</v>
+      <c r="N2" s="5" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F3">
         <v>21840</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="H3" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I3">
         <v>94.1</v>
       </c>
       <c r="J3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="K3">
         <v>21790</v>
       </c>
       <c r="L3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="M3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="N3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
+  <autoFilter ref="$A$1:$N$3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
     <col customWidth="true" max="7" min="1" width="18"/>
@@ -1663,56 +1687,56 @@
   <sheetData>
     <row r="1" ht="30" customHeight="true">
       <c r="A1" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="A2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="5">
+        <v>96.3</v>
+      </c>
+      <c r="D2" s="5">
+        <v>13250</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C2">
-        <v>96.3</v>
-      </c>
-      <c r="D2">
-        <v>13250</v>
-      </c>
-      <c r="E2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G2" t="s">
-        <v>51</v>
+      <c r="F2" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C3">
         <v>92.7</v>
@@ -1721,44 +1745,44 @@
         <v>39120</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4">
+      <c r="A4" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="5">
         <v>91.2</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="5">
         <v>42460</v>
       </c>
-      <c r="E4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4" t="s">
-        <v>51</v>
-      </c>
-      <c r="G4" t="s">
-        <v>51</v>
+      <c r="E4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C5">
         <v>88.4</v>
@@ -1767,395 +1791,543 @@
         <v>48380</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="G5" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="A6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="5">
+        <v>94.1</v>
+      </c>
+      <c r="D6" s="5">
+        <v>21790</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C6">
-        <v>94.1</v>
-      </c>
-      <c r="D6">
-        <v>21790</v>
-      </c>
-      <c r="E6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G6" t="s">
-        <v>51</v>
+      <c r="G6" s="5" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
+  <autoFilter ref="$A$1:$G$6"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="22" min="1" width="18"/>
+    <col customWidth="true" max="27" min="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="true">
       <c r="A1" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>25</v>
+        <v>92</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D2">
+      <c r="A2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="5">
         <v>40230</v>
       </c>
-      <c r="E2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F2" t="s">
-        <v>87</v>
-      </c>
-      <c r="G2" t="s">
-        <v>88</v>
-      </c>
-      <c r="H2" t="s">
-        <v>89</v>
-      </c>
-      <c r="I2" t="s">
-        <v>90</v>
-      </c>
-      <c r="J2" t="s">
-        <v>91</v>
-      </c>
-      <c r="K2" t="s">
-        <v>92</v>
-      </c>
-      <c r="L2" t="s">
-        <v>93</v>
-      </c>
-      <c r="M2">
+      <c r="E2" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="M2" s="5">
         <v>6</v>
       </c>
-      <c r="N2" t="s">
-        <v>92</v>
-      </c>
-      <c r="O2" t="s">
-        <v>92</v>
-      </c>
-      <c r="P2" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>92</v>
-      </c>
-      <c r="R2">
+      <c r="N2" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="R2" s="5">
         <v>220</v>
       </c>
-      <c r="S2" t="s">
-        <v>95</v>
-      </c>
-      <c r="T2" t="s">
-        <v>96</v>
-      </c>
-      <c r="U2" t="s">
-        <v>51</v>
-      </c>
-      <c r="V2" t="s">
-        <v>51</v>
+      <c r="S2" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z2" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA2" s="5" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="D3">
         <v>44700</v>
       </c>
       <c r="E3" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="F3" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="G3" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" t="s">
         <v>101</v>
       </c>
-      <c r="I3" t="s">
-        <v>90</v>
-      </c>
       <c r="J3" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="K3" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="L3" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="M3" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="N3" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="O3" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="P3" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="Q3" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="R3" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="S3" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="T3" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="U3" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="V3" t="s">
-        <v>51</v>
+        <v>35</v>
+      </c>
+      <c r="W3" t="s">
+        <v>35</v>
+      </c>
+      <c r="X3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="A4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D4" s="5">
+        <v>17540</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="K4" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D4">
-        <v>17540</v>
-      </c>
-      <c r="E4" t="s">
-        <v>104</v>
-      </c>
-      <c r="F4" t="s">
-        <v>105</v>
-      </c>
-      <c r="G4" t="s">
-        <v>100</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="L4" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="M4" s="5">
+        <v>0</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="R4" s="5">
+        <v>0</v>
+      </c>
+      <c r="S4" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="I4" t="s">
+      <c r="T4" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="J4" t="s">
-        <v>108</v>
-      </c>
-      <c r="K4" t="s">
-        <v>92</v>
-      </c>
-      <c r="L4" t="s">
-        <v>103</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4" t="s">
-        <v>109</v>
-      </c>
-      <c r="O4" t="s">
-        <v>109</v>
-      </c>
-      <c r="P4" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>109</v>
-      </c>
-      <c r="R4">
-        <v>0</v>
-      </c>
-      <c r="S4" t="s">
-        <v>95</v>
-      </c>
-      <c r="T4" t="s">
-        <v>96</v>
-      </c>
-      <c r="U4" t="s">
-        <v>51</v>
-      </c>
-      <c r="V4" t="s">
-        <v>51</v>
+      <c r="U4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>21790</v>
       </c>
       <c r="E5" t="s">
+        <v>121</v>
+      </c>
+      <c r="F5" t="s">
+        <v>122</v>
+      </c>
+      <c r="G5" t="s">
         <v>111</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" t="s">
+        <v>35</v>
+      </c>
+      <c r="K5" t="s">
+        <v>35</v>
+      </c>
+      <c r="L5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M5" t="s">
+        <v>35</v>
+      </c>
+      <c r="N5" t="s">
+        <v>35</v>
+      </c>
+      <c r="O5" t="s">
+        <v>35</v>
+      </c>
+      <c r="P5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>35</v>
+      </c>
+      <c r="R5" t="s">
+        <v>35</v>
+      </c>
+      <c r="S5" t="s">
         <v>112</v>
       </c>
-      <c r="G5" t="s">
-        <v>100</v>
-      </c>
-      <c r="H5" t="s">
-        <v>101</v>
-      </c>
-      <c r="I5" t="s">
-        <v>101</v>
-      </c>
-      <c r="J5" t="s">
-        <v>101</v>
-      </c>
-      <c r="K5" t="s">
-        <v>101</v>
-      </c>
-      <c r="L5" t="s">
-        <v>101</v>
-      </c>
-      <c r="M5" t="s">
-        <v>101</v>
-      </c>
-      <c r="N5" t="s">
-        <v>101</v>
-      </c>
-      <c r="O5" t="s">
-        <v>101</v>
-      </c>
-      <c r="P5" t="s">
-        <v>101</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>101</v>
-      </c>
-      <c r="R5" t="s">
-        <v>101</v>
-      </c>
-      <c r="S5" t="s">
-        <v>102</v>
-      </c>
       <c r="T5" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="U5" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="V5" t="s">
-        <v>51</v>
+        <v>35</v>
+      </c>
+      <c r="W5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
+  <autoFilter ref="$A$1:$AA$5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="21" min="1" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="true">
+      <c r="A1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+  </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(members): add display-name preferences
</commit_message>
<xml_diff>
--- a/public/downloads/sample-ipace-owner-data.xlsx
+++ b/public/downloads/sample-ipace-owner-data.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Experiences" sheetId="6" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName hidden="true" localSheetId="1" name="_xlnm._FilterDatabase">'Membership'!$A$1:$M$2</definedName>
+    <definedName hidden="true" localSheetId="1" name="_xlnm._FilterDatabase">'Membership'!$A$1:$N$2</definedName>
     <definedName hidden="true" localSheetId="2" name="_xlnm._FilterDatabase">'Vehicles'!$A$1:$N$3</definedName>
     <definedName hidden="true" localSheetId="3" name="_xlnm._FilterDatabase">'SoH History'!$A$1:$G$6</definedName>
     <definedName hidden="true" localSheetId="4" name="_xlnm._FilterDatabase">'Service &amp; Faults'!$A$1:$AA$5</definedName>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
   <si>
     <t>My I-PACE owner data</t>
   </si>
@@ -84,6 +84,9 @@
     <t>Name</t>
   </si>
   <si>
+    <t>Display name</t>
+  </si>
+  <si>
     <t>Country</t>
   </si>
   <si>
@@ -118,6 +121,9 @@
   </si>
   <si>
     <t>Alex Owner</t>
+  </si>
+  <si>
+    <t>Alex</t>
   </si>
   <si>
     <t>United Kingdom</t>
@@ -450,31 +456,31 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <fonts count="5">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="18"/>
+      <color rgb="FFFFFFFF"/>
       <family val="2"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="18"/>
+      <family val="2"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="FF12324A"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF12324A"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF12324A"/>
-    </font>
-    <font>
-      <family val="2"/>
-      <color rgb="FF12324A"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -605,6 +611,11 @@
           <spPr>
             <a:ln cap="rnd" w="25400"/>
           </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr/>
+          </marker>
           <dLbls>
             <spPr/>
             <txPr>
@@ -623,12 +634,6 @@
             <showBubbleSize val="0"/>
             <showLeaderLines val="0"/>
           </dLbls>
-          <marker>
-            <symbol val="circle"/>
-            <size val="6"/>
-            <spPr/>
-          </marker>
-          <invertIfNegative val="0"/>
           <cat>
             <strRef>
               <f>'SoH History'!$B$2:$B$6</f>
@@ -831,6 +836,7 @@
               <f>Events</f>
             </strRef>
           </tx>
+          <invertIfNegative val="0"/>
           <dLbls>
             <spPr/>
             <txPr>
@@ -849,7 +855,6 @@
             <showBubbleSize val="0"/>
             <showLeaderLines val="0"/>
           </dLbls>
-          <invertIfNegative val="0"/>
           <cat>
             <strRef>
               <f>Summary!$J$2:$J$5</f>
@@ -863,7 +868,6 @@
               </numCache>
             </numRef>
           </val>
-          <smooth val="0"/>
         </ser>
         <dLbls>
           <showLegendKey val="0"/>
@@ -1442,7 +1446,7 @@
   <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="13" min="1" width="18"/>
+    <col customWidth="true" max="14" min="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="true">
@@ -1485,50 +1489,56 @@
       <c r="M1" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="N1" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>36</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$M$2"/>
+  <autoFilter ref="$A$1:$N$2"/>
 </worksheet>
 </file>
 
@@ -1542,134 +1552,134 @@
   <sheetData>
     <row r="1" ht="30" customHeight="true">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F2" s="5">
         <v>48520</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I2" s="5">
         <v>88.4</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K2" s="5">
         <v>48380</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F3">
         <v>21840</v>
       </c>
       <c r="G3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I3">
         <v>94.1</v>
       </c>
       <c r="J3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="K3">
         <v>21790</v>
       </c>
       <c r="L3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="N3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1687,33 +1697,33 @@
   <sheetData>
     <row r="1" ht="30" customHeight="true">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C2" s="5">
         <v>96.3</v>
@@ -1722,21 +1732,21 @@
         <v>13250</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C3">
         <v>92.7</v>
@@ -1745,21 +1755,21 @@
         <v>39120</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C4" s="5">
         <v>91.2</v>
@@ -1768,21 +1778,21 @@
         <v>42460</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C5">
         <v>88.4</v>
@@ -1791,21 +1801,21 @@
         <v>48380</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C6" s="5">
         <v>94.1</v>
@@ -1814,13 +1824,13 @@
         <v>21790</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1838,417 +1848,417 @@
   <sheetData>
     <row r="1" ht="30" customHeight="true">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D2" s="5">
         <v>40230</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="M2" s="5">
         <v>6</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P2" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q2" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>103</v>
       </c>
       <c r="R2" s="5">
         <v>220</v>
       </c>
       <c r="S2" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="T2" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Y2" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="AA2" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D3">
         <v>44700</v>
       </c>
       <c r="E3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G3" t="s">
+        <v>113</v>
+      </c>
+      <c r="H3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J3" t="s">
+        <v>104</v>
+      </c>
+      <c r="K3" t="s">
+        <v>105</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>37</v>
+      </c>
+      <c r="O3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>37</v>
+      </c>
+      <c r="R3" t="s">
+        <v>37</v>
+      </c>
+      <c r="S3" t="s">
+        <v>114</v>
+      </c>
+      <c r="T3" t="s">
         <v>109</v>
       </c>
-      <c r="F3" t="s">
-        <v>110</v>
-      </c>
-      <c r="G3" t="s">
-        <v>111</v>
-      </c>
-      <c r="H3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" t="s">
-        <v>101</v>
-      </c>
-      <c r="J3" t="s">
-        <v>102</v>
-      </c>
-      <c r="K3" t="s">
-        <v>103</v>
-      </c>
-      <c r="L3" t="s">
-        <v>35</v>
-      </c>
-      <c r="M3" t="s">
-        <v>35</v>
-      </c>
-      <c r="N3" t="s">
-        <v>35</v>
-      </c>
-      <c r="O3" t="s">
-        <v>35</v>
-      </c>
-      <c r="P3" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>35</v>
-      </c>
-      <c r="R3" t="s">
-        <v>35</v>
-      </c>
-      <c r="S3" t="s">
-        <v>112</v>
-      </c>
-      <c r="T3" t="s">
-        <v>107</v>
-      </c>
       <c r="U3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="V3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="W3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="X3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Y3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Z3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="AA3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D4" s="5">
         <v>17540</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F4" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>113</v>
       </c>
       <c r="M4" s="5">
         <v>0</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="R4" s="5">
         <v>0</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Y4" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Z4" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="AA4" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D5">
         <v>21790</v>
       </c>
       <c r="E5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="I5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="K5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="L5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="O5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="P5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Q5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="R5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="S5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="T5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="U5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="V5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="W5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="X5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Y5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Z5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="AA5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2265,67 +2275,67 @@
   <sheetData>
     <row r="1" ht="30" customHeight="true">
       <c r="A1" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>